<commit_message>
Expand itinerary for all destinations and add kids' booking column
- Morning/afternoon/evening plan for Lisbon, Marrakech, Budapest and Athens
- Blank 'Localizador (meninos)' column in the flights sheet
- E-visa marked done; Ryanair priority note removed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbPxpFjYDQnzNa7KTrLMWP
</commit_message>
<xml_diff>
--- a/Roteiro_Baku_Tbilisi.xlsx
+++ b/Roteiro_Baku_Tbilisi.xlsx
@@ -22,12 +22,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="295">
   <si>
     <t xml:space="preserve">Itinerário de Voos</t>
   </si>
   <si>
-    <t xml:space="preserve">Horários no fuso local de cada aeroporto. Linha amarela = voo ainda não comprado.</t>
+    <t xml:space="preserve">Horários no fuso local de cada aeroporto. Linha amarela = voo ainda não comprado. Coluna lilás = preencher com os localizadores dos meninos.</t>
   </si>
   <si>
     <t xml:space="preserve">Data</t>
@@ -51,6 +51,9 @@
     <t xml:space="preserve">Localizador</t>
   </si>
   <si>
+    <t xml:space="preserve">Localizador (meninos)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Status</t>
   </si>
   <si>
@@ -357,7 +360,7 @@
     <t xml:space="preserve">Proposta de Roteiro: 16/10 a 05/11/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Verde = Azerbaijão/Geórgia (foco do roteiro). Azul = dias de deslocamento.</t>
+    <t xml:space="preserve">Verde = dias de passeio. Azul = dias de deslocamento. Amarelo = item ainda pendente.</t>
   </si>
   <si>
     <t xml:space="preserve">Dia</t>
@@ -366,7 +369,13 @@
     <t xml:space="preserve">Cidade</t>
   </si>
   <si>
-    <t xml:space="preserve">Programação</t>
+    <t xml:space="preserve">Manhã</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noite</t>
   </si>
   <si>
     <t xml:space="preserve">Logística / Observações</t>
@@ -381,7 +390,10 @@
     <t xml:space="preserve">Brasília → São Paulo</t>
   </si>
   <si>
-    <t xml:space="preserve">Deslocamento.</t>
+    <t xml:space="preserve">Voo para São Paulo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Livre.</t>
   </si>
   <si>
     <t xml:space="preserve">AD 6017 BSB 15:55 → CGH 17:40.</t>
@@ -396,15 +408,18 @@
     <t xml:space="preserve">sáb</t>
   </si>
   <si>
-    <t xml:space="preserve">Livre.</t>
-  </si>
-  <si>
     <t xml:space="preserve">dom</t>
   </si>
   <si>
     <t xml:space="preserve">São Paulo → Luanda</t>
   </si>
   <si>
+    <t xml:space="preserve">Ir para GRU (~15:00).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voo noturno.</t>
+  </si>
+  <si>
     <t xml:space="preserve">DT 748 GRU 18:05 → NBJ 06:40 (+1).</t>
   </si>
   <si>
@@ -420,6 +435,12 @@
     <t xml:space="preserve">Conexão em Luanda.</t>
   </si>
   <si>
+    <t xml:space="preserve">Voo para Lisboa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chegada; jantar leve perto do hotel.</t>
+  </si>
+  <si>
     <t xml:space="preserve">DT 652 NBJ 13:00 → LIS 20:35.</t>
   </si>
   <si>
@@ -432,10 +453,16 @@
     <t xml:space="preserve">Lisboa → Marraquexe</t>
   </si>
   <si>
-    <t xml:space="preserve">Dia livre em Lisboa (Alfama, Baixa, Belém).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FR 4390 LIS 22:20 → RAK 22:55. Conferir tamanho da mochila (item pessoal Ryanair ≈ 40×20×25 cm).</t>
+    <t xml:space="preserve">Belém: Mosteiro dos Jerónimos, Torre de Belém, pastéis de Belém.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alfama e Miradouro de Santa Luzia; Baixa e Praça do Comércio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sair ~20:00 para o aeroporto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR 4390 LIS 22:20 → RAK 22:55. Transfer do riad combinado para a chegada noturna.</t>
   </si>
   <si>
     <t xml:space="preserve">Marraquexe</t>
@@ -447,7 +474,16 @@
     <t xml:space="preserve">qua</t>
   </si>
   <si>
-    <t xml:space="preserve">Medina, Praça Jemaa el-Fna, souks, Palácio da Bahia, Jardim Majorelle.</t>
+    <t xml:space="preserve">Jardim Majorelle e Museu Yves Saint Laurent (abre cedo, menos fila).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palácio da Bahia, Túmulos Saadianos e souks da Medina.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Praça Jemaa el-Fna ao pôr do sol; jantar num terraço.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Majorelle exige ingresso online com horário.</t>
   </si>
   <si>
     <t xml:space="preserve">qui</t>
@@ -456,10 +492,16 @@
     <t xml:space="preserve">Marraquexe → Budapeste</t>
   </si>
   <si>
-    <t xml:space="preserve">Manhã: Medersa Ben Youssef e Túmulos Saadianos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">W6 2460 RAK 16:20 → BUD 20:30. Item pessoal Wizz ≈ 40×30×20 cm.</t>
+    <t xml:space="preserve">Medersa Ben Youssef e Le Jardin Secret.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sair ~13:30 para o aeroporto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chegada em Budapeste.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W6 2460 RAK 16:20 → BUD 20:30. Conferir mochila x item pessoal Wizz (≈ 40×30×20 cm).</t>
   </si>
   <si>
     <t xml:space="preserve">Budapeste</t>
@@ -468,22 +510,43 @@
     <t xml:space="preserve">23/10/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Castelo de Buda, Bastião dos Pescadores, Ponte das Correntes, Parlamento; fim de tarde nas Termas Széchenyi.</t>
+    <t xml:space="preserve">Buda: Castelo, Igreja de Matias, Bastião dos Pescadores.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponte das Correntes; visita guiada ao Parlamento.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Termas Széchenyi; jantar no centro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parlamento e Széchenyi: comprar online.</t>
   </si>
   <si>
     <t xml:space="preserve">24/10/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Grande Mercado, Basílica de Santo Estêvão, bairro judeu e ruin bars; cruzeiro noturno no Danúbio.</t>
+    <t xml:space="preserve">Grande Mercado Central; Avenida Andrássy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basílica de Santo Estêvão (vista da cúpula); Sapatos no Danúbio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cruzeiro noturno no Danúbio; ruin bars no bairro judeu (Szimpla Kert).</t>
   </si>
   <si>
     <t xml:space="preserve">Budapeste → Baku</t>
   </si>
   <si>
-    <t xml:space="preserve">Fim de tarde: Bulvar, Cidade Velha (Icherisheher) à noite e Flame Towers iluminadas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">W6 2365 BUD 12:15 → GYD 15:50. Exige e-visa ASAN aprovado.</t>
+    <t xml:space="preserve">Café da manhã; sair ~09:45 para o aeroporto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voo; chegada 15:50.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulvar, Cidade Velha (Icherisheher) e Flame Towers iluminadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W6 2365 BUD 12:15 → GYD 15:50. E-visa ASAN em mãos.</t>
   </si>
   <si>
     <t xml:space="preserve">Baku</t>
@@ -492,7 +555,13 @@
     <t xml:space="preserve">26/10/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Cidade Velha: Torre da Donzela, Palácio dos Shirvanshahs; Museu do Tapete; funicular até o Parque Highland.</t>
+    <t xml:space="preserve">Cidade Velha: Torre da Donzela, Palácio dos Shirvanshahs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Museu do Tapete; funicular até o Parque Highland.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jantar azerbaijano na Cidade Velha.</t>
   </si>
   <si>
     <t xml:space="preserve">Centro Heydar Aliyev costuma fechar às segundas.</t>
@@ -504,7 +573,13 @@
     <t xml:space="preserve">Baku (arredores)</t>
   </si>
   <si>
-    <t xml:space="preserve">Bate-volta: Gobustan (petróglifos, UNESCO) + vulcões de lama; Ateshgah (templo do fogo); Yanar Dag ao pôr do sol.</t>
+    <t xml:space="preserve">Gobustan (petróglifos, UNESCO) + vulcões de lama.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ateshgah (templo do fogo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yanar Dag ao pôr do sol.</t>
   </si>
   <si>
     <t xml:space="preserve">Tour ou motorista privado (dia inteiro).</t>
@@ -513,10 +588,16 @@
     <t xml:space="preserve">Baku → Tbilisi</t>
   </si>
   <si>
-    <t xml:space="preserve">Manhã: Centro Heydar Aliyev; almoço de despedida.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sair ~18:00 para GYD. AZAL GYD 20:50 → TBS 22:00 (PENDENTE DE COMPRA).</t>
+    <t xml:space="preserve">Centro Heydar Aliyev.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Almoço de despedida; sair ~18:00 para GYD.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voo para Tbilisi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AZAL GYD 20:50 → TBS 22:00 (PENDENTE DE COMPRA).</t>
   </si>
   <si>
     <t xml:space="preserve">Tbilisi</t>
@@ -525,7 +606,13 @@
     <t xml:space="preserve">29/10/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Cidade Velha, banhos sulfurosos de Abanotubani, Fortaleza de Narikala (teleférico), Ponte da Paz.</t>
+    <t xml:space="preserve">Cidade Velha e Catedral de Sameba.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banhos sulfurosos de Abanotubani; teleférico até Narikala.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponte da Paz; jantar georgiano com vinho kvevri.</t>
   </si>
   <si>
     <t xml:space="preserve">30/10/2026</t>
@@ -534,19 +621,31 @@
     <t xml:space="preserve">Kazbegi (bate-volta)</t>
   </si>
   <si>
-    <t xml:space="preserve">Estrada Militar Georgiana: Ananuri → mirante de Gudauri → Stepantsminda → Igreja da Trindade de Gergeti.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~3h por trecho. Motorista privado ou tour. Se nevar, trocar com o dia 31.</t>
+    <t xml:space="preserve">Saída ~08:00: Fortaleza de Ananuri; mirante de Gudauri.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stepantsminda e Igreja da Trindade de Gergeti.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retorno a Tbilisi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~3h por trecho. Se nevar, trocar com o dia 31.</t>
   </si>
   <si>
     <t xml:space="preserve">31/10/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Dia reserva para Kazbegi; ou Mtskheta, mercado da Dry Bridge, jantar georgiano.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Late checkout ou manter a noite. Sair ~23:30 para TBS.</t>
+    <t xml:space="preserve">Dia reserva para Kazbegi; ou Mtskheta (Jvari e Svetitskhoveli).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mercado da Dry Bridge; Rua Rustaveli.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jantar; sair ~23:30 para TBS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Late checkout ou manter a noite.</t>
   </si>
   <si>
     <t xml:space="preserve">A bordo / aeroporto</t>
@@ -555,7 +654,13 @@
     <t xml:space="preserve">Tbilisi → Atenas</t>
   </si>
   <si>
-    <t xml:space="preserve">Descanso pela manhã; à tarde Plaka e Anafiotika.</t>
+    <t xml:space="preserve">Chegada 04:15; descanso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plaka e Anafiotika.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jantar em Monastiraki com vista da Acrópole.</t>
   </si>
   <si>
     <t xml:space="preserve">GQ 785 TBS 02:45 → ATH 04:15. Pedir early check-in.</t>
@@ -567,16 +672,28 @@
     <t xml:space="preserve">02/11/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Acrópole + Museu da Acrópole, Ágora Antiga, Monastiraki; pôr do sol no Licabeto.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acrópole cedo para evitar filas.</t>
+    <t xml:space="preserve">Acrópole (primeiro horário) e Museu da Acrópole.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ágora Antiga e Templo de Hefesto; Monastiraki.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pôr do sol no Monte Licabeto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acrópole: ingresso online com horário.</t>
   </si>
   <si>
     <t xml:space="preserve">Atenas → Lisboa → Luanda</t>
   </si>
   <si>
-    <t xml:space="preserve">Tarde livre em Lisboa (~11h de espera).</t>
+    <t xml:space="preserve">Sair ~06:30 para o aeroporto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lisboa: Chiado, Bairro Alto, Elevador de Santa Justa; LX Factory.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sair ~19:30 para o aeroporto.</t>
   </si>
   <si>
     <t xml:space="preserve">A3 720 ATH 08:35 → LIS 11:05; DT 653 LIS 22:30 → NBJ 06:05 (+1).</t>
@@ -585,13 +702,19 @@
     <t xml:space="preserve">Luanda → São Paulo</t>
   </si>
   <si>
-    <t xml:space="preserve">DT 747 NBJ 10:35 → GRU 15:05. Voo seguinte sai de CGH: deslocar GRU → CGH.</t>
+    <t xml:space="preserve">Voo; chegada 15:05.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ir de GRU para perto de CGH.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DT 747 NBJ 10:35 → GRU 15:05.</t>
   </si>
   <si>
     <t xml:space="preserve">São Paulo → Brasília</t>
   </si>
   <si>
-    <t xml:space="preserve">Retorno.</t>
+    <t xml:space="preserve">Voo para Brasília.</t>
   </si>
   <si>
     <t xml:space="preserve">AD 6414 CGH 09:05 → BSB 10:55.</t>
@@ -603,7 +726,7 @@
     <t xml:space="preserve">Pendências</t>
   </si>
   <si>
-    <t xml:space="preserve">Edite apenas a coluna Status (lista suspensa). O resumo abaixo atualiza sozinho.</t>
+    <t xml:space="preserve">Edite apenas a coluna Status (lista suspensa). O resumo abaixo atualiza sozinho. Hospedagens já reservadas: marque Concluído.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -624,46 +747,121 @@
     <t xml:space="preserve">E-visa ASAN (Azerbaijão)</t>
   </si>
   <si>
-    <t xml:space="preserve">Imediato</t>
-  </si>
-  <si>
     <t xml:space="preserve">Alta</t>
   </si>
   <si>
+    <t xml:space="preserve">Concluído</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Já emitido. Levar impresso e no celular.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comprar voo AZAL Baku → Tbilisi (28/10, 20:50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Esta semana</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendente</t>
   </si>
   <si>
-    <t xml:space="preserve">Só pelo site oficial evisa.gov.az. ~US$ 23; prazo padrão de 3 dias úteis (há opção urgente). Embarque para Baku em 25/10.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comprar voo AZAL Baku → Tbilisi (28/10, 20:50)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Esta semana</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cotado a R$ 407 com mala de mão. Trem Baku–Tbilisi indisponível para quem entra com e-visa.</t>
   </si>
   <si>
-    <t xml:space="preserve">Conferir mochila x item pessoal Ryanair e Wizz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se a mochila não couber, incluir Priority na reserva antes do aeroporto.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hospedagem Baku (25 a 28/10, 3 noites)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ficar na Cidade Velha ou perto do Bulvar.</t>
+    <t xml:space="preserve">Conferir mochila x item pessoal Wizz (22/10 e 25/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item pessoal ≈ 40×30×20 cm. Se não couber, incluir WIZZ Priority antes do aeroporto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hospedagem Marraquexe (20 a 22/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riad na Medina; combinar transfer para chegada às 22:55.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hospedagem Budapeste (22 a 25/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distrito V ou VII.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hospedagem Baku (25 a 28/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cidade Velha ou perto do Bulvar.</t>
   </si>
   <si>
     <t xml:space="preserve">Hospedagem Tbilisi (28/10 a 01/11)</t>
   </si>
   <si>
-    <t xml:space="preserve">Chegada ~22:30 no dia 28; saída ~23:30 no dia 31. Negociar late checkout ou manter a noite do dia 31.</t>
+    <t xml:space="preserve">Chegada ~22:30 no dia 28; saída ~23:30 no dia 31. Late checkout ou manter a noite do dia 31.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hospedagem Atenas (01 a 03/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Média</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chegada 04:15 no dia 01: pedir early check-in ou reservar desde 31/10.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pernoite São Paulo (04/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 01/11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega em GRU, sai de CGH: hotel perto de Congonhas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresso Jardim Majorelle (21/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Só online, com horário marcado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visita guiada Parlamento de Budapeste (23/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Esgota com antecedência; escolher horário em inglês ou espanhol.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresso Termas Széchenyi (23/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 23/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baixa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Online sai mais barato; levar chinelo e toalha ou alugar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cruzeiro noturno no Danúbio (24/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 24/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opções de 1h com ou sem jantar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tour Gobustan + Absheron (27/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 25/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tour em grupo ou motorista privado.</t>
   </si>
   <si>
     <t xml:space="preserve">Transporte Kazbegi (30/10)</t>
@@ -672,58 +870,31 @@
     <t xml:space="preserve">Até 28/10</t>
   </si>
   <si>
-    <t xml:space="preserve">Média</t>
-  </si>
-  <si>
     <t xml:space="preserve">Motorista privado (GoTrip/Bolt) ou tour em grupo; dia 31 como reserva.</t>
   </si>
   <si>
-    <t xml:space="preserve">Tour Gobustan + Absheron (27/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Até 25/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tour em grupo ou motorista privado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hospedagem Atenas (01 a 03/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chegada 04:15 no dia 01: pedir early check-in ou reservar desde 31/10.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pernoite São Paulo (04/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Até 01/11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chega em GRU, sai de CGH: hotel perto de Congonhas facilita.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingressos Acrópole (02/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baixa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comprar online com horário marcado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chip / eSIM (Azerbaijão e Geórgia)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eSIM regional Cáucaso ou chip local (Azercell / Magti).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Câmbio: manat (AZN) e lari (GEL)</t>
+    <t xml:space="preserve">Ingresso Acrópole (02/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Online, primeiro horário do dia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chip / eSIM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 22/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eSIM com cobertura em Marrocos, Hungria (UE), Azerbaijão e Geórgia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Câmbio</t>
   </si>
   <si>
     <t xml:space="preserve">Na chegada</t>
   </si>
   <si>
-    <t xml:space="preserve">Sacar no caixa eletrônico do aeroporto; cartão aceito amplamente nas capitais.</t>
+    <t xml:space="preserve">Dirham (MAD) só se obtém no Marrocos; forint (HUF), manat (AZN), lari (GEL) e euro: sacar no caixa eletrônico.</t>
   </si>
   <si>
     <t xml:space="preserve">Concluídas</t>
@@ -816,7 +987,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -831,6 +1002,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFEDE7F6"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFF2F2F2"/>
       </patternFill>
@@ -838,7 +1015,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDDEBF7"/>
-        <bgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFEDE7F6"/>
       </patternFill>
     </fill>
     <fill>
@@ -850,7 +1027,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFEDE7F6"/>
       </patternFill>
     </fill>
   </fills>
@@ -932,28 +1109,16 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -968,11 +1133,23 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1034,7 +1211,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFEDE7F6"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -1252,7 +1429,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -1262,7 +1439,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1275,7 +1453,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1300,431 +1478,450 @@
       <c r="H4" s="3" t="s">
         <v>9</v>
       </c>
+      <c r="I4" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" s="4" t="s">
         <v>17</v>
+      </c>
+      <c r="H5" s="6"/>
+      <c r="I5" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="6"/>
+      <c r="I6" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>17</v>
+      <c r="H7" s="6"/>
+      <c r="I7" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>17</v>
+        <v>37</v>
+      </c>
+      <c r="H8" s="6"/>
+      <c r="I8" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>17</v>
+        <v>44</v>
+      </c>
+      <c r="H9" s="6"/>
+      <c r="I9" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>17</v>
+        <v>50</v>
+      </c>
+      <c r="H10" s="6"/>
+      <c r="I10" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B11" s="7" t="s">
+      <c r="A11" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="B11" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="C11" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="E11" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="F11" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="G11" s="7" t="s">
         <v>57</v>
+      </c>
+      <c r="H11" s="6"/>
+      <c r="I11" s="9" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>17</v>
+        <v>65</v>
+      </c>
+      <c r="H12" s="6"/>
+      <c r="I12" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>17</v>
+        <v>72</v>
+      </c>
+      <c r="H13" s="6"/>
+      <c r="I13" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
+      </c>
+      <c r="H14" s="6"/>
+      <c r="I14" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
+      </c>
+      <c r="H15" s="6"/>
+      <c r="I15" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H16" s="4" t="s">
         <v>17</v>
+      </c>
+      <c r="H16" s="6"/>
+      <c r="I16" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>17</v>
+        <v>93</v>
+      </c>
+      <c r="H17" s="6"/>
+      <c r="I17" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="G18" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>17</v>
+      <c r="H18" s="6"/>
+      <c r="I18" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>17</v>
+        <v>105</v>
+      </c>
+      <c r="H19" s="6"/>
+      <c r="I19" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="G20" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>17</v>
+      <c r="H20" s="6"/>
+      <c r="I20" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H20" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I20" type="list">
       <formula1>"Confirmado,Pendente de compra"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1744,25 +1941,26 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1770,429 +1968,565 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="E5" s="11" t="s">
+      <c r="A5" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="C5" s="11" t="s">
         <v>121</v>
       </c>
+      <c r="D5" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="A6" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="D6" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="C6" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5" t="s">
-        <v>121</v>
+      <c r="E6" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="E7" s="11" t="s">
+      <c r="A7" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="B13" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="C13" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="13" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>154</v>
+      <c r="C14" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>155</v>
+        <v>176</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>154</v>
+        <v>175</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>156</v>
+        <v>177</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>154</v>
+        <v>179</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>160</v>
+        <v>183</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>154</v>
+        <v>185</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>162</v>
+        <v>187</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>164</v>
+        <v>188</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>189</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>165</v>
+        <v>190</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>166</v>
+        <v>193</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>165</v>
+        <v>192</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="E18" s="15"/>
+        <v>194</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>195</v>
+      </c>
       <c r="F18" s="15" t="s">
-        <v>165</v>
+        <v>196</v>
+      </c>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>165</v>
+        <v>201</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="H19" s="15" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>172</v>
+        <v>203</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>165</v>
+        <v>192</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>173</v>
+        <v>204</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>174</v>
+        <v>205</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B21" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="H20" s="15" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>210</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="G21" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="H21" s="15" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="F22" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="G22" s="15" t="s">
+        <v>219</v>
+      </c>
+      <c r="H22" s="15" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="H23" s="12" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="H24" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="C21" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="F21" s="11" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>179</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>185</v>
-      </c>
-      <c r="F23" s="11" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>187</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>121</v>
-      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>189</v>
-      </c>
-      <c r="E25" s="11" t="s">
-        <v>190</v>
-      </c>
-      <c r="F25" s="11" t="s">
-        <v>191</v>
+      <c r="A25" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -2211,7 +2545,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -2224,52 +2558,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>193</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>194</v>
+        <v>235</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>195</v>
+        <v>236</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>196</v>
+        <v>237</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>197</v>
+        <v>238</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>199</v>
+        <v>240</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>200</v>
+        <v>57</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>201</v>
+        <v>241</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>202</v>
+        <v>242</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>203</v>
+        <v>243</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2277,19 +2611,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>204</v>
+        <v>244</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>205</v>
+        <v>245</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>201</v>
+        <v>241</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>202</v>
+        <v>246</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>206</v>
+        <v>247</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2297,19 +2631,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>207</v>
+        <v>248</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>208</v>
+        <v>249</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>201</v>
+        <v>241</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>202</v>
+        <v>246</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>209</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2317,39 +2651,39 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>210</v>
+        <v>251</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>205</v>
+        <v>252</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>201</v>
+        <v>241</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>202</v>
+        <v>246</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>212</v>
+        <v>254</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>201</v>
+        <v>241</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>202</v>
+        <v>246</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>213</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2357,39 +2691,39 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>214</v>
+        <v>256</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>216</v>
+        <v>245</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>241</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>202</v>
+        <v>246</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>218</v>
+        <v>258</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>216</v>
+        <v>245</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>241</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>202</v>
+        <v>246</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>220</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2397,19 +2731,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>221</v>
+        <v>260</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>205</v>
+        <v>245</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>216</v>
+        <v>261</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>202</v>
+        <v>246</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>222</v>
+        <v>262</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2417,19 +2751,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>223</v>
+        <v>263</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>224</v>
+        <v>264</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>216</v>
+        <v>261</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>202</v>
+        <v>246</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>225</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2437,19 +2771,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>226</v>
+        <v>266</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>227</v>
+        <v>252</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>241</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>202</v>
+        <v>246</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>228</v>
+        <v>267</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2457,19 +2791,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>229</v>
+        <v>268</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>219</v>
+        <v>249</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>227</v>
+        <v>261</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>202</v>
+        <v>246</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>230</v>
+        <v>269</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2477,59 +2811,179 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>231</v>
+        <v>270</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>232</v>
+        <v>271</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>227</v>
+        <v>272</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>202</v>
+        <v>246</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>233</v>
+        <v>273</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="B18" s="18" t="n">
-        <f aca="false">COUNTIF(E5:E16,"Concluído")</f>
+      <c r="A18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="17" t="s">
+        <v>291</v>
+      </c>
+      <c r="B24" s="18" t="n">
+        <f aca="false">COUNTIF(E5:E22,"Concluído")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="17" t="s">
+        <v>292</v>
+      </c>
+      <c r="B25" s="18" t="n">
+        <f aca="false">COUNTIF(E5:E22,"Em andamento")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
-        <v>235</v>
-      </c>
-      <c r="B19" s="18" t="n">
-        <f aca="false">COUNTIF(E5:E16,"Em andamento")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
-        <v>236</v>
-      </c>
-      <c r="B20" s="18" t="n">
-        <f aca="false">COUNTIF(E5:E16,"Pendente")</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17" t="s">
-        <v>237</v>
-      </c>
-      <c r="B21" s="19" t="n">
-        <f aca="false">IFERROR(B18/COUNTA(B5:B16),0)</f>
-        <v>0</v>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="17" t="s">
+        <v>293</v>
+      </c>
+      <c r="B26" s="18" t="n">
+        <f aca="false">COUNTIF(E5:E22,"Pendente")</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="17" t="s">
+        <v>294</v>
+      </c>
+      <c r="B27" s="19" t="n">
+        <f aca="false">IFERROR(B24/COUNTA(B5:B22),0)</f>
+        <v>0.0555555555555556</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A5:F16">
+  <conditionalFormatting sqref="A5:F22">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$E5="Concluído"</formula>
     </cfRule>
@@ -2538,7 +2992,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E16" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E22" type="list">
       <formula1>"Pendente,Em andamento,Concluído"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Add hostel booking sheet for all stops except Lisbon
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbPxpFjYDQnzNa7KTrLMWP
</commit_message>
<xml_diff>
--- a/Roteiro_Baku_Tbilisi.xlsx
+++ b/Roteiro_Baku_Tbilisi.xlsx
@@ -9,8 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Voos" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Roteiro" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Pendências" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Hospedagem" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Roteiro" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Pendências" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="322">
   <si>
     <t xml:space="preserve">Itinerário de Voos</t>
   </si>
@@ -357,6 +358,117 @@
     <t xml:space="preserve">Voo pendente: cotação de R$ 407 (1 item pessoal + 1 mala de mão, sem despachada), direto, 1h10. Número do voo a confirmar na compra.</t>
   </si>
   <si>
+    <t xml:space="preserve">Hospedagem (hostels)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lilás = preencher após reservar. Noites e total calculados automaticamente. Lisboa não incluída.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cidade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noites</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chegada / saída</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Região sugerida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hostel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor total (R$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observações</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marraquexe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega 22:55 (20/10) / sai ~13:30 (22/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medina, perto da Jemaa el-Fna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URGENTE: chegada hoje à noite. Pedir transfer do aeroporto; carro não entra na Medina.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budapeste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega 20:30 (22/10) / sai ~09:45 (25/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distrito VII (bairro judeu) ou V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Região dos ruin bars; boa ligação de metrô.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baku</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega ~16:30 (25/10) / sai ~18:00 (28/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cidade Velha (Icherisheher) ou Nizami</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedir para guardar as mochilas no dia 28 até a saída para o aeroporto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tbilisi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega ~22:30 (28/10) / sai ~23:30 (31/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cidade Velha ou Sololaki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 noites: garante cama até sair para o voo das 02:45. Confirmar check-in tardio. Ponto de saída para Kazbegi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atenas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega 04:15 (01/11) / sai ~06:30 (03/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monastiraki, Psyri ou Plaka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-in a partir de 31/10 garante cama ao chegar de madrugada. Alternativa: 01 a 03/11 e pedir early check-in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">São Paulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega 15:05 em GRU (04/11) / voo CGH 09:05 (05/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perto de Congonhas (Moema, Campo Belo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Só se não houver onde ficar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
     <t xml:space="preserve">Proposta de Roteiro: 16/10 a 05/11/2026</t>
   </si>
   <si>
@@ -366,9 +478,6 @@
     <t xml:space="preserve">Dia</t>
   </si>
   <si>
-    <t xml:space="preserve">Cidade</t>
-  </si>
-  <si>
     <t xml:space="preserve">Manhã</t>
   </si>
   <si>
@@ -399,9 +508,6 @@
     <t xml:space="preserve">AD 6017 BSB 15:55 → CGH 17:40.</t>
   </si>
   <si>
-    <t xml:space="preserve">São Paulo</t>
-  </si>
-  <si>
     <t xml:space="preserve">17/10/2026</t>
   </si>
   <si>
@@ -462,10 +568,7 @@
     <t xml:space="preserve">Sair ~20:00 para o aeroporto.</t>
   </si>
   <si>
-    <t xml:space="preserve">FR 4390 LIS 22:20 → RAK 22:55. Transfer do riad combinado para a chegada noturna.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marraquexe</t>
+    <t xml:space="preserve">FR 4390 LIS 22:20 → RAK 22:55. Transfer do hostel combinado para a chegada noturna.</t>
   </si>
   <si>
     <t xml:space="preserve">21/10/2026</t>
@@ -504,9 +607,6 @@
     <t xml:space="preserve">W6 2460 RAK 16:20 → BUD 20:30. Conferir mochila x item pessoal Wizz (≈ 40×30×20 cm).</t>
   </si>
   <si>
-    <t xml:space="preserve">Budapeste</t>
-  </si>
-  <si>
     <t xml:space="preserve">23/10/2026</t>
   </si>
   <si>
@@ -549,9 +649,6 @@
     <t xml:space="preserve">W6 2365 BUD 12:15 → GYD 15:50. E-visa ASAN em mãos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Baku</t>
-  </si>
-  <si>
     <t xml:space="preserve">26/10/2026</t>
   </si>
   <si>
@@ -600,9 +697,6 @@
     <t xml:space="preserve">AZAL GYD 20:50 → TBS 22:00 (PENDENTE DE COMPRA).</t>
   </si>
   <si>
-    <t xml:space="preserve">Tbilisi</t>
-  </si>
-  <si>
     <t xml:space="preserve">29/10/2026</t>
   </si>
   <si>
@@ -666,9 +760,6 @@
     <t xml:space="preserve">GQ 785 TBS 02:45 → ATH 04:15. Pedir early check-in.</t>
   </si>
   <si>
-    <t xml:space="preserve">Atenas</t>
-  </si>
-  <si>
     <t xml:space="preserve">02/11/2026</t>
   </si>
   <si>
@@ -726,7 +817,7 @@
     <t xml:space="preserve">Pendências</t>
   </si>
   <si>
-    <t xml:space="preserve">Edite apenas a coluna Status (lista suspensa). O resumo abaixo atualiza sozinho. Hospedagens já reservadas: marque Concluído.</t>
+    <t xml:space="preserve">Edite apenas a coluna Status (lista suspensa). O resumo abaixo atualiza sozinho.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -741,9 +832,6 @@
     <t xml:space="preserve">Prioridade</t>
   </si>
   <si>
-    <t xml:space="preserve">Observações</t>
-  </si>
-  <si>
     <t xml:space="preserve">E-visa ASAN (Azerbaijão)</t>
   </si>
   <si>
@@ -762,9 +850,6 @@
     <t xml:space="preserve">Esta semana</t>
   </si>
   <si>
-    <t xml:space="preserve">Pendente</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cotado a R$ 407 com mala de mão. Trem Baku–Tbilisi indisponível para quem entra com e-visa.</t>
   </si>
   <si>
@@ -777,54 +862,60 @@
     <t xml:space="preserve">Item pessoal ≈ 40×30×20 cm. Se não couber, incluir WIZZ Priority antes do aeroporto.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hospedagem Marraquexe (20 a 22/10)</t>
+    <t xml:space="preserve">Reservar hostel Marraquexe (20 a 22/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOJE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chegada 22:55: combinar transfer, carro não entra na Medina. Ver aba Hospedagem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar hostel Budapeste (22 a 25/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ver aba Hospedagem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar hostel Baku (25 a 28/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 23/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar hostel Tbilisi (28/10 a 01/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 25/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-in ~22:30 no dia 28. Ver aba Hospedagem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar hostel Atenas (31/10 a 03/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 28/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Média</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar pernoite São Paulo (04 a 05/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 01/11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se não houver onde ficar. Ver aba Hospedagem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresso Jardim Majorelle (21/10)</t>
   </si>
   <si>
     <t xml:space="preserve">Hoje</t>
   </si>
   <si>
-    <t xml:space="preserve">Riad na Medina; combinar transfer para chegada às 22:55.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hospedagem Budapeste (22 a 25/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distrito V ou VII.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hospedagem Baku (25 a 28/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cidade Velha ou perto do Bulvar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hospedagem Tbilisi (28/10 a 01/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chegada ~22:30 no dia 28; saída ~23:30 no dia 31. Late checkout ou manter a noite do dia 31.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hospedagem Atenas (01 a 03/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Média</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chegada 04:15 no dia 01: pedir early check-in ou reservar desde 31/10.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pernoite São Paulo (04/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Até 01/11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chega em GRU, sai de CGH: hotel perto de Congonhas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingresso Jardim Majorelle (21/10)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Só online, com horário marcado.</t>
   </si>
   <si>
@@ -837,9 +928,6 @@
     <t xml:space="preserve">Ingresso Termas Széchenyi (23/10)</t>
   </si>
   <si>
-    <t xml:space="preserve">Até 23/10</t>
-  </si>
-  <si>
     <t xml:space="preserve">Baixa</t>
   </si>
   <si>
@@ -858,16 +946,10 @@
     <t xml:space="preserve">Tour Gobustan + Absheron (27/10)</t>
   </si>
   <si>
-    <t xml:space="preserve">Até 25/10</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tour em grupo ou motorista privado.</t>
   </si>
   <si>
     <t xml:space="preserve">Transporte Kazbegi (30/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Até 28/10</t>
   </si>
   <si>
     <t xml:space="preserve">Motorista privado (GoTrip/Bolt) ou tour em grupo; dia 31 como reserva.</t>
@@ -913,10 +995,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="0%"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="166" formatCode="&quot;R$ &quot;#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="General"/>
+    <numFmt numFmtId="168" formatCode="0%"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -1014,6 +1098,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFEDE7F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFDDEBF7"/>
         <bgColor rgb="FFEDE7F6"/>
       </patternFill>
@@ -1022,12 +1112,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
         <bgColor rgb="FFDDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFEDE7F6"/>
       </patternFill>
     </fill>
   </fills>
@@ -1080,7 +1164,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1121,16 +1205,32 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1145,19 +1245,27 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1941,6 +2049,297 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="52"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>46317</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <f aca="false">C5-B5</f>
+        <v>2</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="K5" s="13" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <f aca="false">C6-B6</f>
+        <v>3</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>46320</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <f aca="false">C7-B7</f>
+        <v>3</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>46327</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <f aca="false">C8-B8</f>
+        <v>4</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>46329</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <f aca="false">C9-B9</f>
+        <v>3</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>46330</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>46331</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <f aca="false">C10-B10</f>
+        <v>1</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="14" t="n">
+        <f aca="false">SUM(D5:D10)</f>
+        <v>16</v>
+      </c>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="16" t="n">
+        <f aca="false">SUM(I5:I10)</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="J5:J10">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>OR($J5="Reservado",$J5="Pago")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>$J5="Pendente"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J10" type="list">
+      <formula1>"Pendente,Reservado,Pago"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:H25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1955,12 +2354,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1968,565 +2367,565 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>114</v>
-      </c>
       <c r="D4" s="3" t="s">
-        <v>115</v>
+        <v>151</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>117</v>
+        <v>153</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>119</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="D5" s="12" t="s">
+      <c r="B5" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="D5" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="H5" s="19" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="H7" s="19" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>173</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="H8" s="19" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>179</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>181</v>
+      </c>
+      <c r="H9" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="F5" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="B6" s="10" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>184</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="F10" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>187</v>
+      </c>
+      <c r="H10" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>190</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>192</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>193</v>
+      </c>
+      <c r="H11" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="C6" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="F7" s="12" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="20" t="s">
+        <v>194</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>127</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>196</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>197</v>
+      </c>
+      <c r="G12" s="22" t="s">
+        <v>198</v>
+      </c>
+      <c r="H12" s="22" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="20" t="s">
+        <v>199</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>127</v>
+      </c>
+      <c r="D13" s="22" t="s">
+        <v>200</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>202</v>
+      </c>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>203</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>204</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>205</v>
+      </c>
+      <c r="F14" s="22" t="s">
+        <v>206</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>207</v>
+      </c>
+      <c r="H14" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="G7" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="H7" s="12" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="C8" s="11" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="B15" s="20" t="s">
+        <v>169</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>209</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>211</v>
+      </c>
+      <c r="G15" s="22" t="s">
+        <v>212</v>
+      </c>
+      <c r="H15" s="22" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>214</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>215</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>216</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>217</v>
+      </c>
+      <c r="G16" s="22" t="s">
+        <v>218</v>
+      </c>
+      <c r="H16" s="22" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>219</v>
+      </c>
+      <c r="D17" s="22" t="s">
+        <v>220</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>222</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="H17" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="D8" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="G8" s="12" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="20" t="s">
+        <v>224</v>
+      </c>
+      <c r="B18" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="D18" s="22" t="s">
+        <v>225</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>226</v>
+      </c>
+      <c r="F18" s="22" t="s">
+        <v>227</v>
+      </c>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="20" t="s">
+        <v>228</v>
+      </c>
+      <c r="B19" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>229</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>230</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>231</v>
+      </c>
+      <c r="F19" s="22" t="s">
+        <v>232</v>
+      </c>
+      <c r="G19" s="22" t="s">
+        <v>233</v>
+      </c>
+      <c r="H19" s="22" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="B20" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>235</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>236</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>237</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>238</v>
+      </c>
+      <c r="H20" s="22" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="D21" s="22" t="s">
+        <v>241</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>242</v>
+      </c>
+      <c r="F21" s="22" t="s">
+        <v>243</v>
+      </c>
+      <c r="G21" s="22" t="s">
+        <v>244</v>
+      </c>
+      <c r="H21" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="H8" s="12" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="D9" s="15" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="20" t="s">
+        <v>245</v>
+      </c>
+      <c r="B22" s="20" t="s">
+        <v>169</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="D22" s="22" t="s">
+        <v>246</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>247</v>
+      </c>
+      <c r="F22" s="22" t="s">
+        <v>248</v>
+      </c>
+      <c r="G22" s="22" t="s">
+        <v>249</v>
+      </c>
+      <c r="H22" s="22" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>250</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>252</v>
+      </c>
+      <c r="F23" s="19" t="s">
+        <v>253</v>
+      </c>
+      <c r="G23" s="19" t="s">
+        <v>254</v>
+      </c>
+      <c r="H23" s="19" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>255</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="E24" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="F24" s="19" t="s">
+        <v>257</v>
+      </c>
+      <c r="G24" s="19" t="s">
+        <v>258</v>
+      </c>
+      <c r="H24" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="E9" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="F9" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="G9" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="H9" s="15" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="E10" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="F10" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="G10" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="H10" s="15" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="G11" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="H11" s="15" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>161</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="F12" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="G12" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="H12" s="15" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>168</v>
-      </c>
-      <c r="F13" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>171</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="F14" s="15" t="s">
-        <v>173</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>174</v>
-      </c>
-      <c r="H14" s="15" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="C15" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>177</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="F15" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G15" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H15" s="15" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="D16" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="F16" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="G16" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="H16" s="15" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>187</v>
-      </c>
-      <c r="D17" s="15" t="s">
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="E17" s="15" t="s">
-        <v>189</v>
-      </c>
-      <c r="F17" s="15" t="s">
-        <v>190</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>191</v>
-      </c>
-      <c r="H17" s="15" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
-        <v>193</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>192</v>
-      </c>
-      <c r="D18" s="15" t="s">
-        <v>194</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>195</v>
-      </c>
-      <c r="F18" s="15" t="s">
-        <v>196</v>
-      </c>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
-        <v>197</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>198</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>199</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>200</v>
-      </c>
-      <c r="F19" s="15" t="s">
-        <v>201</v>
-      </c>
-      <c r="G19" s="15" t="s">
-        <v>202</v>
-      </c>
-      <c r="H19" s="15" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>192</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>204</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>205</v>
-      </c>
-      <c r="F20" s="15" t="s">
-        <v>206</v>
-      </c>
-      <c r="G20" s="15" t="s">
-        <v>207</v>
-      </c>
-      <c r="H20" s="15" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>209</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>210</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>211</v>
-      </c>
-      <c r="F21" s="15" t="s">
-        <v>212</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>213</v>
-      </c>
-      <c r="H21" s="15" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
-        <v>215</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>214</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>216</v>
-      </c>
-      <c r="E22" s="15" t="s">
-        <v>217</v>
-      </c>
-      <c r="F22" s="15" t="s">
-        <v>218</v>
-      </c>
-      <c r="G22" s="15" t="s">
-        <v>219</v>
-      </c>
-      <c r="H22" s="15" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>220</v>
-      </c>
-      <c r="D23" s="12" t="s">
-        <v>221</v>
-      </c>
-      <c r="E23" s="12" t="s">
-        <v>222</v>
-      </c>
-      <c r="F23" s="12" t="s">
-        <v>223</v>
-      </c>
-      <c r="G23" s="12" t="s">
-        <v>224</v>
-      </c>
-      <c r="H23" s="12" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>225</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="E24" s="12" t="s">
-        <v>226</v>
-      </c>
-      <c r="F24" s="12" t="s">
-        <v>227</v>
-      </c>
-      <c r="G24" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="H24" s="12" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="C25" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>230</v>
-      </c>
-      <c r="E25" s="12" t="s">
+      <c r="C25" s="18" t="s">
+        <v>259</v>
+      </c>
+      <c r="D25" s="19" t="s">
+        <v>260</v>
+      </c>
+      <c r="E25" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="F25" s="12" t="s">
+      <c r="F25" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="G25" s="12" t="s">
-        <v>231</v>
-      </c>
-      <c r="H25" s="12" t="s">
-        <v>232</v>
+      <c r="G25" s="19" t="s">
+        <v>261</v>
+      </c>
+      <c r="H25" s="19" t="s">
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -2540,7 +2939,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -2558,32 +2957,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>233</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>234</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>235</v>
+        <v>265</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>236</v>
+        <v>266</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>237</v>
+        <v>267</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>238</v>
+        <v>268</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>239</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2591,19 +2990,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>240</v>
+        <v>269</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D5" s="16" t="s">
-        <v>241</v>
+      <c r="D5" s="23" t="s">
+        <v>270</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2611,19 +3010,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>244</v>
+        <v>273</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>241</v>
+        <v>274</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>270</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>247</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2631,19 +3030,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>248</v>
+        <v>276</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>241</v>
+        <v>277</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>270</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>250</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2651,19 +3050,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>251</v>
+        <v>279</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>241</v>
+        <v>280</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>270</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>253</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2671,19 +3070,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>254</v>
+        <v>282</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>241</v>
+        <v>277</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>270</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>255</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2691,39 +3090,39 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>256</v>
+        <v>284</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>241</v>
+        <v>285</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>270</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>258</v>
+        <v>286</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>241</v>
+        <v>287</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>270</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>259</v>
+        <v>288</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2731,19 +3130,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>260</v>
+        <v>289</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>245</v>
+        <v>290</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>261</v>
+        <v>291</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>262</v>
+        <v>283</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2751,19 +3150,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>263</v>
+        <v>292</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>264</v>
+        <v>293</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>261</v>
+        <v>291</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>265</v>
+        <v>294</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2771,19 +3170,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>266</v>
+        <v>295</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="D14" s="16" t="s">
-        <v>241</v>
+        <v>296</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>270</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>267</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2791,19 +3190,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>268</v>
+        <v>298</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>249</v>
+        <v>277</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>261</v>
+        <v>291</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>269</v>
+        <v>299</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2811,19 +3210,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>270</v>
+        <v>300</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2831,19 +3230,19 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>274</v>
+        <v>303</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>275</v>
+        <v>304</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>276</v>
+        <v>305</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2851,19 +3250,19 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>277</v>
+        <v>306</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>261</v>
+        <v>291</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>279</v>
+        <v>307</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2871,19 +3270,19 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>280</v>
+        <v>308</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>261</v>
+        <v>291</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>282</v>
+        <v>309</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2891,19 +3290,19 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>283</v>
+        <v>310</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>264</v>
+        <v>293</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>261</v>
+        <v>291</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>284</v>
+        <v>311</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2911,19 +3310,19 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>285</v>
+        <v>312</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>286</v>
+        <v>313</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>287</v>
+        <v>314</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2931,53 +3330,53 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>288</v>
+        <v>315</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>289</v>
+        <v>316</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>290</v>
+        <v>317</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="s">
-        <v>291</v>
-      </c>
-      <c r="B24" s="18" t="n">
+      <c r="A24" s="14" t="s">
+        <v>318</v>
+      </c>
+      <c r="B24" s="24" t="n">
         <f aca="false">COUNTIF(E5:E22,"Concluído")</f>
         <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17" t="s">
-        <v>292</v>
-      </c>
-      <c r="B25" s="18" t="n">
+      <c r="A25" s="14" t="s">
+        <v>319</v>
+      </c>
+      <c r="B25" s="24" t="n">
         <f aca="false">COUNTIF(E5:E22,"Em andamento")</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="s">
-        <v>293</v>
-      </c>
-      <c r="B26" s="18" t="n">
+      <c r="A26" s="14" t="s">
+        <v>320</v>
+      </c>
+      <c r="B26" s="24" t="n">
         <f aca="false">COUNTIF(E5:E22,"Pendente")</f>
         <v>17</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17" t="s">
-        <v>294</v>
-      </c>
-      <c r="B27" s="19" t="n">
+      <c r="A27" s="14" t="s">
+        <v>321</v>
+      </c>
+      <c r="B27" s="25" t="n">
         <f aca="false">IFERROR(B24/COUNTA(B5:B22),0)</f>
         <v>0.0555555555555556</v>
       </c>

</xml_diff>

<commit_message>
Remove Wizz Air backpack/priority check from itinerary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbPxpFjYDQnzNa7KTrLMWP
</commit_message>
<xml_diff>
--- a/Roteiro_Baku_Tbilisi.xlsx
+++ b/Roteiro_Baku_Tbilisi.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="320">
   <si>
     <t xml:space="preserve">Itinerário de Voos</t>
   </si>
@@ -604,7 +604,7 @@
     <t xml:space="preserve">Chegada em Budapeste.</t>
   </si>
   <si>
-    <t xml:space="preserve">W6 2460 RAK 16:20 → BUD 20:30. Conferir mochila x item pessoal Wizz (≈ 40×30×20 cm).</t>
+    <t xml:space="preserve">W6 2460 RAK 16:20 → BUD 20:30.</t>
   </si>
   <si>
     <t xml:space="preserve">23/10/2026</t>
@@ -853,25 +853,19 @@
     <t xml:space="preserve">Cotado a R$ 407 com mala de mão. Trem Baku–Tbilisi indisponível para quem entra com e-visa.</t>
   </si>
   <si>
-    <t xml:space="preserve">Conferir mochila x item pessoal Wizz (22/10 e 25/10)</t>
+    <t xml:space="preserve">Reservar hostel Marraquexe (20 a 22/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOJE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chegada 22:55: combinar transfer, carro não entra na Medina. Ver aba Hospedagem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar hostel Budapeste (22 a 25/10)</t>
   </si>
   <si>
     <t xml:space="preserve">21/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Item pessoal ≈ 40×30×20 cm. Se não couber, incluir WIZZ Priority antes do aeroporto.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reservar hostel Marraquexe (20 a 22/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HOJE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chegada 22:55: combinar transfer, carro não entra na Medina. Ver aba Hospedagem.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reservar hostel Budapeste (22 a 25/10)</t>
   </si>
   <si>
     <t xml:space="preserve">Ver aba Hospedagem.</t>
@@ -2944,7 +2938,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -3073,7 +3067,7 @@
         <v>282</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="D9" s="23" t="s">
         <v>270</v>
@@ -3082,7 +3076,7 @@
         <v>125</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3102,7 +3096,7 @@
         <v>125</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3110,19 +3104,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>270</v>
+        <v>288</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>289</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>125</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3130,19 +3124,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>289</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>291</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>125</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3150,19 +3144,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>291</v>
+        <v>294</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>270</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>125</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3170,13 +3164,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>296</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>270</v>
+        <v>280</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>289</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>125</v>
@@ -3193,16 +3187,16 @@
         <v>298</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>125</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3210,19 +3204,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>285</v>
+        <v>302</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>125</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3230,13 +3224,13 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>304</v>
+        <v>285</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>125</v>
@@ -3253,10 +3247,10 @@
         <v>306</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>125</v>
@@ -3273,10 +3267,10 @@
         <v>308</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>125</v>
@@ -3293,96 +3287,76 @@
         <v>310</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>293</v>
+        <v>311</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>125</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>125</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="5" t="s">
         <v>315</v>
       </c>
-      <c r="C22" s="4" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
         <v>316</v>
       </c>
-      <c r="D22" s="4" t="s">
-        <v>301</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>317</v>
+      <c r="B23" s="24" t="n">
+        <f aca="false">COUNTIF(E5:E21,"Concluído")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B24" s="24" t="n">
-        <f aca="false">COUNTIF(E5:E22,"Concluído")</f>
-        <v>1</v>
+        <f aca="false">COUNTIF(E5:E21,"Em andamento")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B25" s="24" t="n">
-        <f aca="false">COUNTIF(E5:E22,"Em andamento")</f>
-        <v>0</v>
+        <f aca="false">COUNTIF(E5:E21,"Pendente")</f>
+        <v>16</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>320</v>
-      </c>
-      <c r="B26" s="24" t="n">
-        <f aca="false">COUNTIF(E5:E22,"Pendente")</f>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14" t="s">
-        <v>321</v>
-      </c>
-      <c r="B27" s="25" t="n">
-        <f aca="false">IFERROR(B24/COUNTA(B5:B22),0)</f>
-        <v>0.0555555555555556</v>
+        <v>319</v>
+      </c>
+      <c r="B26" s="25" t="n">
+        <f aca="false">IFERROR(B23/COUNTA(B5:B21),0)</f>
+        <v>0.0588235294117647</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A5:F22">
+  <conditionalFormatting sqref="A5:F21">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$E5="Concluído"</formula>
     </cfRule>
@@ -3391,7 +3365,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E22" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E21" type="list">
       <formula1>"Pendente,Em andamento,Concluído"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Add Marrakech riad booking and flag missing second night
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbPxpFjYDQnzNa7KTrLMWP
</commit_message>
<xml_diff>
--- a/Roteiro_Baku_Tbilisi.xlsx
+++ b/Roteiro_Baku_Tbilisi.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="330">
   <si>
     <t xml:space="preserve">Itinerário de Voos</t>
   </si>
@@ -385,7 +385,7 @@
     <t xml:space="preserve">Hostel</t>
   </si>
   <si>
-    <t xml:space="preserve">Valor total (R$)</t>
+    <t xml:space="preserve">Valor total</t>
   </si>
   <si>
     <t xml:space="preserve">Observações</t>
@@ -394,16 +394,31 @@
     <t xml:space="preserve">Marraquexe</t>
   </si>
   <si>
-    <t xml:space="preserve">Chega 22:55 (20/10) / sai ~13:30 (22/10)</t>
+    <t xml:space="preserve">Chega 22:55 (20/10)</t>
   </si>
   <si>
     <t xml:space="preserve">Medina, perto da Jemaa el-Fna</t>
   </si>
   <si>
+    <t xml:space="preserve">Riad Hna Ben Saleh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6552802435</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riad Hna Ben Saleh, Derb Bouaanane, Ben Saleh nº 44, Medina. Quarto família, 4 adultos, café incluído. PAGAMENTO SÓ EM DINHEIRO (MAD). Não reembolsável. Avisar horário de chegada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sai ~13:30 (22/10)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendente</t>
   </si>
   <si>
-    <t xml:space="preserve">URGENTE: chegada hoje à noite. Pedir transfer do aeroporto; carro não entra na Medina.</t>
+    <t xml:space="preserve">URGENTE: a reserva atual cobre só 1 noite. Tentar estender no mesmo riad (21 a 22/10).</t>
   </si>
   <si>
     <t xml:space="preserve">Budapeste</t>
@@ -469,6 +484,9 @@
     <t xml:space="preserve">Total</t>
   </si>
   <si>
+    <t xml:space="preserve">Valores em moedas diferentes: não somados.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Proposta de Roteiro: 16/10 a 05/11/2026</t>
   </si>
   <si>
@@ -568,7 +586,7 @@
     <t xml:space="preserve">Sair ~20:00 para o aeroporto.</t>
   </si>
   <si>
-    <t xml:space="preserve">FR 4390 LIS 22:20 → RAK 22:55. Transfer do hostel combinado para a chegada noturna.</t>
+    <t xml:space="preserve">FR 4390 LIS 22:20 → RAK 22:55. Riad Hna Ben Saleh (Derb Bouaanane, Ben Saleh nº 44): avisar horário de chegada; pagamento só em dinheiro (MAD).</t>
   </si>
   <si>
     <t xml:space="preserve">21/10/2026</t>
@@ -586,7 +604,7 @@
     <t xml:space="preserve">Praça Jemaa el-Fna ao pôr do sol; jantar num terraço.</t>
   </si>
   <si>
-    <t xml:space="preserve">Majorelle exige ingresso online com horário.</t>
+    <t xml:space="preserve">Majorelle exige ingresso online com horário. Pernoite 21/10 ainda sem reserva.</t>
   </si>
   <si>
     <t xml:space="preserve">qui</t>
@@ -853,13 +871,28 @@
     <t xml:space="preserve">Cotado a R$ 407 com mala de mão. Trem Baku–Tbilisi indisponível para quem entra com e-visa.</t>
   </si>
   <si>
-    <t xml:space="preserve">Reservar hostel Marraquexe (20 a 22/10)</t>
+    <t xml:space="preserve">Hospedagem Marraquexe 20 a 21/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riad Hna Ben Saleh, reserva Booking 6552802435. Pagamento só em dinheiro (MAD).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar 2ª noite Marraquexe (21 a 22/10)</t>
   </si>
   <si>
     <t xml:space="preserve">HOJE</t>
   </si>
   <si>
-    <t xml:space="preserve">Chegada 22:55: combinar transfer, carro não entra na Medina. Ver aba Hospedagem.</t>
+    <t xml:space="preserve">Reserva atual cobre só 1 noite. Tentar estender no mesmo riad.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sacar dirham (MAD) para pagar o riad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Na chegada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€ 84,97 pagos em dinheiro na moeda local; sacar no caixa eletrônico do aeroporto de Marraquexe.</t>
   </si>
   <si>
     <t xml:space="preserve">Reservar hostel Budapeste (22 a 25/10)</t>
@@ -965,9 +998,6 @@
   </si>
   <si>
     <t xml:space="preserve">Câmbio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Na chegada</t>
   </si>
   <si>
     <t xml:space="preserve">Dirham (MAD) só se obtém no Marrocos; forint (HUF), manat (AZN), lari (GEL) e euro: sacar no caixa eletrônico.</t>
@@ -989,12 +1019,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="166" formatCode="&quot;R$ &quot;#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="General"/>
-    <numFmt numFmtId="168" formatCode="0%"/>
+    <numFmt numFmtId="166" formatCode="&quot;€ &quot;#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="&quot;R$ &quot;#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="General"/>
+    <numFmt numFmtId="169" formatCode="0%"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -1158,7 +1189,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1215,6 +1246,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1223,7 +1258,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1255,11 +1290,11 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2043,7 +2078,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -2068,7 +2103,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>113</v>
       </c>
@@ -2103,7 +2138,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
         <v>122</v>
       </c>
@@ -2111,11 +2146,11 @@
         <v>46315</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">C5-B5</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>123</v>
@@ -2123,189 +2158,224 @@
       <c r="F5" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="12"/>
+      <c r="G5" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="I5" s="12" t="n">
+        <v>84.97</v>
+      </c>
       <c r="J5" s="4" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B6" s="11" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C6" s="11" t="n">
         <v>46317</v>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>46320</v>
       </c>
       <c r="D6" s="4" t="n">
         <f aca="false">C6-B6</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
-      <c r="I6" s="12"/>
+      <c r="I6" s="14"/>
       <c r="J6" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="K6" s="5" t="s">
         <v>130</v>
+      </c>
+      <c r="K6" s="13" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B7" s="11" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C7" s="11" t="n">
         <v>46320</v>
-      </c>
-      <c r="C7" s="11" t="n">
-        <v>46323</v>
       </c>
       <c r="D7" s="4" t="n">
         <f aca="false">C7-B7</f>
         <v>3</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
-      <c r="I7" s="12"/>
+      <c r="I7" s="14"/>
       <c r="J7" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B8" s="11" t="n">
+        <v>46320</v>
+      </c>
+      <c r="C8" s="11" t="n">
         <v>46323</v>
-      </c>
-      <c r="C8" s="11" t="n">
-        <v>46327</v>
       </c>
       <c r="D8" s="4" t="n">
         <f aca="false">C8-B8</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
-      <c r="I8" s="12"/>
+      <c r="I8" s="14"/>
       <c r="J8" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B9" s="11" t="n">
-        <v>46326</v>
+        <v>46323</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>46329</v>
+        <v>46327</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">C9-B9</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
-      <c r="I9" s="12"/>
+      <c r="I9" s="14"/>
       <c r="J9" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B10" s="11" t="n">
-        <v>46330</v>
+        <v>46326</v>
       </c>
       <c r="C10" s="11" t="n">
-        <v>46331</v>
+        <v>46329</v>
       </c>
       <c r="D10" s="4" t="n">
         <f aca="false">C10-B10</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
-      <c r="I10" s="12"/>
+      <c r="I10" s="14"/>
       <c r="J10" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="14" t="n">
-        <f aca="false">SUM(D5:D10)</f>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>46330</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>46331</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <f aca="false">C11-B11</f>
+        <v>1</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="15" t="n">
+        <f aca="false">SUM(D5:D11)</f>
         <v>16</v>
       </c>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="16" t="n">
-        <f aca="false">SUM(I5:I10)</f>
-        <v>0</v>
-      </c>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="17" t="s">
+        <v>153</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J5:J10">
+  <conditionalFormatting sqref="J5:J11">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>OR($J5="Reservado",$J5="Pago")</formula>
     </cfRule>
@@ -2314,7 +2384,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J10" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J11" type="list">
       <formula1>"Pendente,Reservado,Pago"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2348,12 +2418,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2361,565 +2431,565 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>113</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="17" t="s">
-        <v>156</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>157</v>
-      </c>
-      <c r="D5" s="19" t="s">
+      <c r="B5" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="D5" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="E5" s="19" t="s">
-        <v>158</v>
-      </c>
-      <c r="F5" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="G5" s="19" t="s">
-        <v>160</v>
-      </c>
-      <c r="H5" s="19" t="s">
-        <v>143</v>
+      <c r="E5" s="20" t="s">
+        <v>164</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="H5" s="20" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
-        <v>161</v>
-      </c>
-      <c r="B6" s="17" t="s">
+      <c r="A6" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>172</v>
+      </c>
+      <c r="G7" s="20" t="s">
+        <v>173</v>
+      </c>
+      <c r="H7" s="20" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>177</v>
+      </c>
+      <c r="E8" s="20" t="s">
+        <v>178</v>
+      </c>
+      <c r="F8" s="20" t="s">
+        <v>179</v>
+      </c>
+      <c r="G8" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="H8" s="20" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>182</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>183</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="G10" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>194</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>196</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="G11" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="B12" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>143</v>
-      </c>
-      <c r="D6" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="E6" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="F6" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>164</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="G7" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="H7" s="19" t="s">
+      <c r="C12" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>201</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>202</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="G12" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="B13" s="21" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="17" t="s">
+      <c r="C13" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>208</v>
+      </c>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="21" t="s">
         <v>169</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>170</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>171</v>
-      </c>
-      <c r="E8" s="19" t="s">
-        <v>172</v>
-      </c>
-      <c r="F8" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="G8" s="19" t="s">
+      <c r="C14" s="22" t="s">
+        <v>209</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>210</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>211</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>212</v>
+      </c>
+      <c r="G14" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21" t="s">
+        <v>214</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>215</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>216</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>217</v>
+      </c>
+      <c r="G15" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="H15" s="23" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="s">
+        <v>219</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>182</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>220</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>222</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>223</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>224</v>
+      </c>
+      <c r="H16" s="23" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>225</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>226</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>227</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>228</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="H17" s="23" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="s">
+        <v>230</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>194</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>231</v>
+      </c>
+      <c r="E18" s="23" t="s">
+        <v>232</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>233</v>
+      </c>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="s">
+        <v>234</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>235</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>237</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>238</v>
+      </c>
+      <c r="G19" s="23" t="s">
+        <v>239</v>
+      </c>
+      <c r="H19" s="23" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>241</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>242</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>243</v>
+      </c>
+      <c r="G20" s="23" t="s">
+        <v>244</v>
+      </c>
+      <c r="H20" s="23" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>169</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>246</v>
+      </c>
+      <c r="D21" s="23" t="s">
+        <v>247</v>
+      </c>
+      <c r="E21" s="23" t="s">
+        <v>248</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>249</v>
+      </c>
+      <c r="G21" s="23" t="s">
+        <v>250</v>
+      </c>
+      <c r="H21" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21" t="s">
+        <v>251</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>252</v>
+      </c>
+      <c r="E22" s="23" t="s">
+        <v>253</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>254</v>
+      </c>
+      <c r="G22" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="H22" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>257</v>
+      </c>
+      <c r="E23" s="20" t="s">
+        <v>258</v>
+      </c>
+      <c r="F23" s="20" t="s">
+        <v>259</v>
+      </c>
+      <c r="G23" s="20" t="s">
+        <v>260</v>
+      </c>
+      <c r="H23" s="20" t="s">
         <v>174</v>
       </c>
-      <c r="H8" s="19" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>176</v>
-      </c>
-      <c r="C9" s="21" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>261</v>
+      </c>
+      <c r="D24" s="20" t="s">
         <v>177</v>
       </c>
-      <c r="D9" s="22" t="s">
-        <v>178</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>179</v>
-      </c>
-      <c r="F9" s="22" t="s">
-        <v>180</v>
-      </c>
-      <c r="G9" s="22" t="s">
-        <v>181</v>
-      </c>
-      <c r="H9" s="22" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
-        <v>182</v>
-      </c>
-      <c r="B10" s="20" t="s">
-        <v>183</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="D10" s="22" t="s">
-        <v>184</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>185</v>
-      </c>
-      <c r="F10" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="G10" s="22" t="s">
-        <v>187</v>
-      </c>
-      <c r="H10" s="22" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>188</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>189</v>
-      </c>
-      <c r="D11" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="E11" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="F11" s="22" t="s">
-        <v>192</v>
-      </c>
-      <c r="G11" s="22" t="s">
-        <v>193</v>
-      </c>
-      <c r="H11" s="22" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
+      <c r="E24" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="F24" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="G24" s="20" t="s">
+        <v>264</v>
+      </c>
+      <c r="H24" s="20" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="B12" s="20" t="s">
-        <v>156</v>
-      </c>
-      <c r="C12" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="D12" s="22" t="s">
-        <v>195</v>
-      </c>
-      <c r="E12" s="22" t="s">
-        <v>196</v>
-      </c>
-      <c r="F12" s="22" t="s">
-        <v>197</v>
-      </c>
-      <c r="G12" s="22" t="s">
-        <v>198</v>
-      </c>
-      <c r="H12" s="22" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
-        <v>199</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>162</v>
-      </c>
-      <c r="C13" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="D13" s="22" t="s">
-        <v>200</v>
-      </c>
-      <c r="E13" s="22" t="s">
-        <v>201</v>
-      </c>
-      <c r="F13" s="22" t="s">
-        <v>202</v>
-      </c>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="20" t="s">
-        <v>163</v>
-      </c>
-      <c r="C14" s="21" t="s">
-        <v>203</v>
-      </c>
-      <c r="D14" s="22" t="s">
-        <v>204</v>
-      </c>
-      <c r="E14" s="22" t="s">
-        <v>205</v>
-      </c>
-      <c r="F14" s="22" t="s">
-        <v>206</v>
-      </c>
-      <c r="G14" s="22" t="s">
-        <v>207</v>
-      </c>
-      <c r="H14" s="22" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>169</v>
-      </c>
-      <c r="C15" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="D15" s="22" t="s">
-        <v>209</v>
-      </c>
-      <c r="E15" s="22" t="s">
-        <v>210</v>
-      </c>
-      <c r="F15" s="22" t="s">
-        <v>211</v>
-      </c>
-      <c r="G15" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="H15" s="22" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
-        <v>213</v>
-      </c>
-      <c r="B16" s="20" t="s">
-        <v>176</v>
-      </c>
-      <c r="C16" s="21" t="s">
-        <v>214</v>
-      </c>
-      <c r="D16" s="22" t="s">
-        <v>215</v>
-      </c>
-      <c r="E16" s="22" t="s">
-        <v>216</v>
-      </c>
-      <c r="F16" s="22" t="s">
-        <v>217</v>
-      </c>
-      <c r="G16" s="22" t="s">
-        <v>218</v>
-      </c>
-      <c r="H16" s="22" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="B17" s="20" t="s">
-        <v>183</v>
-      </c>
-      <c r="C17" s="21" t="s">
-        <v>219</v>
-      </c>
-      <c r="D17" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="E17" s="22" t="s">
-        <v>221</v>
-      </c>
-      <c r="F17" s="22" t="s">
-        <v>222</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>223</v>
-      </c>
-      <c r="H17" s="22" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20" t="s">
-        <v>224</v>
-      </c>
-      <c r="B18" s="20" t="s">
-        <v>188</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="D18" s="22" t="s">
-        <v>225</v>
-      </c>
-      <c r="E18" s="22" t="s">
-        <v>226</v>
-      </c>
-      <c r="F18" s="22" t="s">
-        <v>227</v>
-      </c>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="s">
-        <v>228</v>
-      </c>
-      <c r="B19" s="20" t="s">
-        <v>156</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>229</v>
-      </c>
-      <c r="D19" s="22" t="s">
-        <v>230</v>
-      </c>
-      <c r="E19" s="22" t="s">
-        <v>231</v>
-      </c>
-      <c r="F19" s="22" t="s">
-        <v>232</v>
-      </c>
-      <c r="G19" s="22" t="s">
-        <v>233</v>
-      </c>
-      <c r="H19" s="22" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="20" t="s">
-        <v>234</v>
-      </c>
-      <c r="B20" s="20" t="s">
-        <v>162</v>
-      </c>
-      <c r="C20" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="D20" s="22" t="s">
-        <v>235</v>
-      </c>
-      <c r="E20" s="22" t="s">
-        <v>236</v>
-      </c>
-      <c r="F20" s="22" t="s">
-        <v>237</v>
-      </c>
-      <c r="G20" s="22" t="s">
-        <v>238</v>
-      </c>
-      <c r="H20" s="22" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="B21" s="20" t="s">
-        <v>163</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>240</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>241</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>242</v>
-      </c>
-      <c r="F21" s="22" t="s">
-        <v>243</v>
-      </c>
-      <c r="G21" s="22" t="s">
-        <v>244</v>
-      </c>
-      <c r="H21" s="22" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="20" t="s">
-        <v>245</v>
-      </c>
-      <c r="B22" s="20" t="s">
-        <v>169</v>
-      </c>
-      <c r="C22" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="D22" s="22" t="s">
-        <v>246</v>
-      </c>
-      <c r="E22" s="22" t="s">
-        <v>247</v>
-      </c>
-      <c r="F22" s="22" t="s">
-        <v>248</v>
-      </c>
-      <c r="G22" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="H22" s="22" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="B23" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>250</v>
-      </c>
-      <c r="D23" s="19" t="s">
-        <v>251</v>
-      </c>
-      <c r="E23" s="19" t="s">
-        <v>252</v>
-      </c>
-      <c r="F23" s="19" t="s">
-        <v>253</v>
-      </c>
-      <c r="G23" s="19" t="s">
-        <v>254</v>
-      </c>
-      <c r="H23" s="19" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="B24" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>255</v>
-      </c>
-      <c r="D24" s="19" t="s">
-        <v>171</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>256</v>
-      </c>
-      <c r="F24" s="19" t="s">
-        <v>257</v>
-      </c>
-      <c r="G24" s="19" t="s">
-        <v>258</v>
-      </c>
-      <c r="H24" s="19" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="B25" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="C25" s="18" t="s">
-        <v>259</v>
-      </c>
-      <c r="D25" s="19" t="s">
-        <v>260</v>
-      </c>
-      <c r="E25" s="19" t="s">
+      <c r="C25" s="19" t="s">
+        <v>265</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>266</v>
+      </c>
+      <c r="E25" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="F25" s="19" t="s">
+      <c r="F25" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="G25" s="19" t="s">
-        <v>261</v>
-      </c>
-      <c r="H25" s="19" t="s">
-        <v>262</v>
+      <c r="G25" s="20" t="s">
+        <v>267</v>
+      </c>
+      <c r="H25" s="20" t="s">
+        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -2938,7 +3008,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -2951,26 +3021,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>10</v>
@@ -2984,19 +3054,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D5" s="23" t="s">
-        <v>270</v>
+      <c r="D5" s="24" t="s">
+        <v>276</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3004,39 +3074,39 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="D6" s="23" t="s">
-        <v>270</v>
+        <v>280</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>276</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="24" t="s">
         <v>276</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="D7" s="23" t="s">
-        <v>270</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>125</v>
-      </c>
       <c r="F7" s="5" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3044,39 +3114,39 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>270</v>
+        <v>285</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>276</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>270</v>
+        <v>288</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>276</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3084,19 +3154,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>285</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>270</v>
+        <v>291</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>276</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3104,19 +3174,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>288</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>289</v>
+        <v>294</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>276</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3124,19 +3194,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>291</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>289</v>
+        <v>296</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>276</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3144,19 +3214,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>270</v>
+        <v>299</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>300</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3164,19 +3234,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>280</v>
+        <v>302</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>289</v>
+        <v>300</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3184,19 +3254,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>299</v>
+        <v>305</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>276</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3204,19 +3274,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3224,19 +3294,19 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>289</v>
+        <v>310</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3244,19 +3314,19 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>288</v>
+        <v>313</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>289</v>
+        <v>310</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3264,19 +3334,19 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>289</v>
+        <v>300</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3284,79 +3354,119 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
-        <v>316</v>
-      </c>
-      <c r="B23" s="24" t="n">
-        <f aca="false">COUNTIF(E5:E21,"Concluído")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
-        <v>317</v>
-      </c>
-      <c r="B24" s="24" t="n">
-        <f aca="false">COUNTIF(E5:E21,"Em andamento")</f>
+        <v>320</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="B25" s="25" t="n">
+        <f aca="false">COUNTIF(E5:E23,"Concluído")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="15" t="s">
+        <v>327</v>
+      </c>
+      <c r="B26" s="25" t="n">
+        <f aca="false">COUNTIF(E5:E23,"Em andamento")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
-        <v>318</v>
-      </c>
-      <c r="B25" s="24" t="n">
-        <f aca="false">COUNTIF(E5:E21,"Pendente")</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="s">
-        <v>319</v>
-      </c>
-      <c r="B26" s="25" t="n">
-        <f aca="false">IFERROR(B23/COUNTA(B5:B21),0)</f>
-        <v>0.0588235294117647</v>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="15" t="s">
+        <v>328</v>
+      </c>
+      <c r="B27" s="25" t="n">
+        <f aca="false">COUNTIF(E5:E23,"Pendente")</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="15" t="s">
+        <v>329</v>
+      </c>
+      <c r="B28" s="26" t="n">
+        <f aca="false">IFERROR(B25/COUNTA(B5:B23),0)</f>
+        <v>0.105263157894737</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A5:F21">
+  <conditionalFormatting sqref="A5:F23">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$E5="Concluído"</formula>
     </cfRule>
@@ -3365,7 +3475,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E21" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E23" type="list">
       <formula1>"Pendente,Em andamento,Concluído"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Mark eSIM for PT/GR/HU/MA as done; keep Caucasus coverage pending
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbPxpFjYDQnzNa7KTrLMWP
</commit_message>
<xml_diff>
--- a/Roteiro_Baku_Tbilisi.xlsx
+++ b/Roteiro_Baku_Tbilisi.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="331">
   <si>
     <t xml:space="preserve">Itinerário de Voos</t>
   </si>
@@ -988,13 +988,16 @@
     <t xml:space="preserve">Online, primeiro horário do dia.</t>
   </si>
   <si>
-    <t xml:space="preserve">Chip / eSIM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Até 22/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eSIM com cobertura em Marrocos, Hungria (UE), Azerbaijão e Geórgia.</t>
+    <t xml:space="preserve">eSIM Portugal, Grécia, Hungria e Marrocos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Já contratado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eSIM ou chip Azerbaijão e Geórgia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não cobertos pelo eSIM atual. Opções: eSIM regional (Airalo, Holafly etc.) ou chip local na chegada (Azercell em Baku, Magti em Tbilisi).</t>
   </si>
   <si>
     <t xml:space="preserve">Câmbio</t>
@@ -3008,7 +3011,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -3397,16 +3400,16 @@
         <v>321</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>322</v>
+        <v>57</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>310</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>130</v>
+        <v>277</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3414,28 +3417,39 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>130</v>
       </c>
       <c r="F23" s="5" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="s">
+      <c r="C24" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F24" s="5" t="s">
         <v>326</v>
-      </c>
-      <c r="B25" s="25" t="n">
-        <f aca="false">COUNTIF(E5:E23,"Concluído")</f>
-        <v>2</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3443,8 +3457,8 @@
         <v>327</v>
       </c>
       <c r="B26" s="25" t="n">
-        <f aca="false">COUNTIF(E5:E23,"Em andamento")</f>
-        <v>0</v>
+        <f aca="false">COUNTIF(E5:E24,"Concluído")</f>
+        <v>3</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3452,21 +3466,30 @@
         <v>328</v>
       </c>
       <c r="B27" s="25" t="n">
-        <f aca="false">COUNTIF(E5:E23,"Pendente")</f>
-        <v>17</v>
+        <f aca="false">COUNTIF(E5:E24,"Em andamento")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
         <v>329</v>
       </c>
-      <c r="B28" s="26" t="n">
-        <f aca="false">IFERROR(B25/COUNTA(B5:B23),0)</f>
-        <v>0.105263157894737</v>
+      <c r="B28" s="25" t="n">
+        <f aca="false">COUNTIF(E5:E24,"Pendente")</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="15" t="s">
+        <v>330</v>
+      </c>
+      <c r="B29" s="26" t="n">
+        <f aca="false">IFERROR(B26/COUNTA(B5:B24),0)</f>
+        <v>0.15</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A5:F23">
+  <conditionalFormatting sqref="A5:F24">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$E5="Concluído"</formula>
     </cfRule>
@@ -3475,7 +3498,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E23" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E24" type="list">
       <formula1>"Pendente,Em andamento,Concluído"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>